<commit_message>
Scrub corporate identity from Excel report templates
Tier-1 (text-only, no formula impact) anonymisation of the four
workbooks in Report samples/:
- Company name POLIMA FOREST BINTULU SDN. BHD. -> GREENACRE PLANTATIONS
- Registration no. 749886-W -> 000000-X
- Estate LADANG BATANG KAYAN -> DEMO ESTATE
- docProps + threaded-comment author registry (Acc Dept / KEVIN CHAN,
  account token) -> Demo
- Leaked local paths E:\KEVIN\... (workbook absPath + externalLink rels)
  -> E:\DEMO\...

Per-gang worksheet tab names (real worker first-names wired into
formulas/charts) are intentionally left for an Excel-validated rename;
README known-limitation note updated to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Report samples/Spraying Maintenance 2025.xlsx
+++ b/Report samples/Spraying Maintenance 2025.xlsx
@@ -72,13 +72,13 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2036" uniqueCount="81">
   <si>
-    <t>POLIMA FOREST BINTULU SDN. BHD.  (Company No. 749886-W)</t>
+    <t>GREENACRE PLANTATIONS SDN. BHD.  (Company No. 000000-X)</t>
   </si>
   <si>
     <t>ESTATE MONTHLY REPORT</t>
   </si>
   <si>
-    <t>LADANG BATANG KAYAN</t>
+    <t>DEMO ESTATE</t>
   </si>
   <si>
     <t>GLYPHOSATE SPRAYING SELECT</t>

</xml_diff>